<commit_message>
adding missing figures and statistics for STOR scenario
</commit_message>
<xml_diff>
--- a/1_REVUB_code/control_file.xlsx
+++ b/1_REVUB_code/control_file.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/2_REVUB_control_file/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/1_REVUB_code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2055" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64BD26A8-091D-4642-BCBE-86970532CE4D}"/>
+  <xr:revisionPtr revIDLastSave="2060" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C86516A-7444-4FD3-BF0F-CBC942719BE9}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="735" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
   </bookViews>
@@ -732,43 +732,6 @@
     <t>Figure7_on</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">set to 1 to plot regulated reservoir release statistics [see worksheet </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Plot release rules (single HPP)]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">, or to 0 to turn off </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[Note: currently only available for BAL]</t>
-    </r>
-  </si>
-  <si>
     <t>Figure8_on</t>
   </si>
   <si>
@@ -776,32 +739,6 @@
   </si>
   <si>
     <t>Figure9_on</t>
-  </si>
-  <si>
-    <r>
-      <t>set to 1 to plot operational regime statistics, or to 0 to turn off [</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Note: currently only available for BAL</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>]</t>
-    </r>
   </si>
   <si>
     <t>plot_rules_month</t>
@@ -1845,6 +1782,77 @@
   </si>
   <si>
     <t>[name 3]</t>
+  </si>
+  <si>
+    <t>set to 1 to plot operational regime statistics, or to 0 to turn off</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">set to 1 to plot regulated reservoir release statistics [see </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_rules_month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_rules_hr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> below</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, or to 0 to turn off</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -2470,31 +2478,31 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
   </sheetData>
@@ -2526,13 +2534,13 @@
         <v>13</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="E2" s="4" t="s">
         <v>225</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.35">
@@ -2585,7 +2593,7 @@
         <v>16</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="10" spans="1:5" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
@@ -2593,7 +2601,7 @@
         <v>108</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2601,7 +2609,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2609,7 +2617,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="3" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2617,7 +2625,7 @@
         <v>17</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2625,7 +2633,7 @@
         <v>18</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2633,7 +2641,7 @@
         <v>19</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -2641,7 +2649,7 @@
         <v>22</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2655,7 +2663,7 @@
         <v>23</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2669,7 +2677,7 @@
         <v>24</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2683,7 +2691,7 @@
         <v>29</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="23" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2691,7 +2699,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="24" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2699,7 +2707,7 @@
         <v>26</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2707,7 +2715,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2715,7 +2723,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2731,7 +2739,7 @@
         <v>33</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="29" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2900,10 +2908,10 @@
     </row>
     <row r="50" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="B50" s="1" t="s">
         <v>200</v>
-      </c>
-      <c r="B50" s="1" t="s">
-        <v>202</v>
       </c>
     </row>
     <row r="51" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2917,7 +2925,7 @@
         <v>59</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="53" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2933,7 +2941,7 @@
         <v>61</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="55" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2941,7 +2949,7 @@
         <v>62</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="56" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -3000,10 +3008,10 @@
     </row>
     <row r="63" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>201</v>
-      </c>
-      <c r="B63" s="1" t="s">
-        <v>203</v>
       </c>
     </row>
   </sheetData>
@@ -3028,13 +3036,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>208</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -3044,7 +3052,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B3" s="20"/>
       <c r="C3" s="20"/>
@@ -3069,18 +3077,18 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B6" s="22">
         <v>0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="20"/>
@@ -3102,7 +3110,7 @@
         <v>0</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -3110,7 +3118,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="21" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -3139,7 +3147,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="21" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>
@@ -3152,7 +3160,7 @@
         <v>1000</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
@@ -3163,7 +3171,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -3174,12 +3182,12 @@
         <v>0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="21" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
@@ -3192,7 +3200,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -3245,13 +3253,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>208</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -3377,54 +3385,54 @@
       </c>
       <c r="B15" s="23"/>
       <c r="C15" t="s">
-        <v>141</v>
+        <v>227</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B16" s="23"/>
       <c r="C16" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B17" s="23"/>
       <c r="C17" t="s">
-        <v>145</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B18" s="23"/>
       <c r="C18" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B20" s="13" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="21" spans="1:3" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
       <c r="B22" s="13" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="23" spans="1:3" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -3452,75 +3460,75 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>209</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B2" s="13" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="3" spans="1:15" s="19" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B5" s="13" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B6" s="23"/>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B8" s="13" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B9" s="22"/>
       <c r="C9" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B11" s="13" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="B12" s="22"/>
       <c r="C12" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B14" s="13" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.35">
       <c r="B15" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="D15" s="14" t="s">
         <v>159</v>
-      </c>
-      <c r="C15" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="D15" s="14" t="s">
-        <v>161</v>
       </c>
       <c r="E15" s="14"/>
       <c r="F15" s="14"/>
@@ -3529,25 +3537,25 @@
     </row>
     <row r="16" spans="1:15" s="12" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="B16" s="22"/>
       <c r="O16" s="15"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B18" s="13" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B19" s="14" t="s">
+        <v>157</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>159</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>160</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>161</v>
       </c>
       <c r="E19" s="14"/>
       <c r="F19" s="14"/>
@@ -3556,17 +3564,17 @@
     </row>
     <row r="20" spans="1:8" s="22" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B22" s="13" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="B23" s="22"/>
       <c r="C23" t="s">
@@ -3575,7 +3583,7 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B24" s="22"/>
       <c r="C24" t="s">
@@ -3584,7 +3592,7 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B25" s="22"/>
       <c r="C25" t="s">
@@ -3593,7 +3601,7 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B26" s="22"/>
       <c r="C26" t="s">
@@ -3602,25 +3610,25 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B27" s="22"/>
       <c r="C27" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B28" s="16"/>
       <c r="C28" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B29" s="23"/>
       <c r="C29" t="s">
@@ -3629,11 +3637,11 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B30" s="23"/>
       <c r="C30" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding extra error warnings + improving user flexibility on lateral inflow
</commit_message>
<xml_diff>
--- a/1_REVUB_code/control_file.xlsx
+++ b/1_REVUB_code/control_file.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://vub-my.sharepoint.com/personal/sebastian_sterl_vub_be/Documents/Documenten/VUB Work Files/REVUB code repo/1_REVUB_code/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2060" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2C86516A-7444-4FD3-BF0F-CBC942719BE9}"/>
+  <xr:revisionPtr revIDLastSave="2063" documentId="13_ncr:1_{3E75B3F6-DB26-4BD5-A9C7-B5D5CA9FF346}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E3F97BC7-252F-4AD4-B3A3-99518A1E2FC6}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="735" xr2:uid="{B27AEA38-A928-4B6A-AF9B-7A28216807AA}"/>
   </bookViews>
@@ -891,38 +891,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[leave empty if unsure - only in case of cascade calculations]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets (use the "inflow" workbook) from which to pull data on </t>
-    </r>
-    <r>
-      <rPr>
-        <u/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>lateral</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> inflow to a downstream cascade plant (hourly flow in </t>
+      <t>[leave empty for zeros]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (precipitation flux in </t>
     </r>
     <r>
       <rPr>
@@ -933,7 +912,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>m^3/s</t>
+      <t>kg/m^2/s</t>
     </r>
     <r>
       <rPr>
@@ -967,7 +946,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (precipitation flux in </t>
+      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (evaporation flux in </t>
     </r>
     <r>
       <rPr>
@@ -1012,7 +991,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (evaporation flux in </t>
+      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data on prescribed (environmental/irrigation) outflow (hourly in </t>
     </r>
     <r>
       <rPr>
@@ -1023,7 +1002,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>kg/m^2/s</t>
+      <t>m^3/s</t>
     </r>
     <r>
       <rPr>
@@ -1047,17 +1026,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[leave empty for zeros]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data on prescribed (environmental/irrigation) outflow (hourly in </t>
+      <t>[leave empty if scenario has no solar]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (hourly solar CF as </t>
     </r>
     <r>
       <rPr>
@@ -1068,17 +1047,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>m^3/s</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>; hours in rows, years in columns)</t>
+      <t>fraction</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>/percentage; hours in rows, years in columns)</t>
     </r>
   </si>
   <si>
@@ -1092,17 +1071,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[leave empty if scenario has no solar]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (hourly solar CF as </t>
+      <t>[leave empty if scenario has no wind]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (hourly wind CF as </t>
     </r>
     <r>
       <rPr>
@@ -1137,17 +1116,17 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[leave empty if scenario has no wind]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (hourly wind CF as </t>
+      <t>[leave empty in calibration run]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (hourly load </t>
     </r>
     <r>
       <rPr>
@@ -1158,17 +1137,92 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>fraction</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>/percentage; hours in rows, years in columns)</t>
+      <t xml:space="preserve">normalised </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>to a mean of unity)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">name of corresponding worksheet in the "data" Excel sheets from which to pull data (first column: volume in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>m^3</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; second: surface area in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>m^2</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">; third: head in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>m</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
     </r>
   </si>
   <si>
@@ -1182,17 +1236,29 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>[leave empty in calibration run]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets from which to pull data (hourly load </t>
+      <t>[leave empty for scenarios without solar/wind]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> fraction of solar in the solar/wind portfolio</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">installed capacity in </t>
     </r>
     <r>
       <rPr>
@@ -1203,29 +1269,19 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">normalised </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>to a mean of unity)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">name of corresponding worksheet in the "data" Excel sheets from which to pull data (first column: volume in </t>
+      <t>MW</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">maximum lake volume in </t>
     </r>
     <r>
       <rPr>
@@ -1238,15 +1294,17 @@
       </rPr>
       <t>m^3</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; second: surface area in </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">maximum lake area in </t>
     </r>
     <r>
       <rPr>
@@ -1259,15 +1317,17 @@
       </rPr>
       <t>m^2</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">; third: head in </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">maximum head in </t>
     </r>
     <r>
       <rPr>
@@ -1280,16 +1340,136 @@
       </rPr>
       <t>m</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">maximum discharge (total of all turbines) in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>m^3/s</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">turbine efficiency as fraction </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[note: power factor can be included here]</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">lower lake volume in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>m^3</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">pump capacity in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>MW</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">pump maximum discharge in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>m^3/s</t>
+    </r>
+  </si>
+  <si>
+    <t>tables_on</t>
+  </si>
+  <si>
+    <t>set to 1 to output key time series in Excel format</t>
+  </si>
+  <si>
+    <t>tables_on_multiple</t>
+  </si>
+  <si>
+    <t>f_init_BAL_opt</t>
+  </si>
+  <si>
+    <t>f_init_STOR_opt</t>
   </si>
   <si>
     <r>
@@ -1297,245 +1477,23 @@
         <b/>
         <i/>
         <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[leave empty for scenarios without solar/wind]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> fraction of solar in the solar/wind portfolio</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">installed capacity in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MW</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">maximum lake volume in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>m^3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">maximum lake area in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>m^2</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">maximum head in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>m</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">maximum discharge (total of all turbines) in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>m^3/s</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">turbine efficiency as fraction </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[note: power factor can be included here]</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">lower lake volume in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>m^3</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">pump capacity in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>MW</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">pump maximum discharge in </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>m^3/s</t>
-    </r>
-  </si>
-  <si>
-    <t>tables_on</t>
-  </si>
-  <si>
-    <t>set to 1 to output key time series in Excel format</t>
-  </si>
-  <si>
-    <t>tables_on_multiple</t>
-  </si>
-  <si>
-    <t>f_init_BAL_opt</t>
-  </si>
-  <si>
-    <t>f_init_STOR_opt</t>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[only use if already known from previous run]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The optimal value in the range of the ELCC for BAL</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1558,7 +1516,276 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> The optimal value in the range of the ELCC for BAL</t>
+      <t xml:space="preserve"> The optimal value in the range of the ELCC for STOR</t>
+    </r>
+  </si>
+  <si>
+    <t>path_inputs</t>
+  </si>
+  <si>
+    <t>path_outputs</t>
+  </si>
+  <si>
+    <t>path to folder with input data sheets</t>
+  </si>
+  <si>
+    <t>path where output will be located</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>parameter</t>
+  </si>
+  <si>
+    <t>explanation</t>
+  </si>
+  <si>
+    <t>value(s)</t>
+  </si>
+  <si>
+    <t>path</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>simulation period</t>
+  </si>
+  <si>
+    <t>simulation settings</t>
+  </si>
+  <si>
+    <t>physical constants</t>
+  </si>
+  <si>
+    <t>simulation accuracy</t>
+  </si>
+  <si>
+    <t>years_skip</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">this parameter allows to skip the first </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">year_skip </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>years of the entered data (default: 0)</t>
+    </r>
+  </si>
+  <si>
+    <t>miscellaneous simulation parameters</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">represents number of years of filling as threshold for determining </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>f_reg</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> if left unspecified by user (see sheet "Hydropower plant parameters"). Default/recommended is unity, so</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> f_reg </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>represents the fraction of annual mean inflow that would take exactly one year to fill reservoir.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">When </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>min(Psi)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (eq. S21) is lower than this threshold, no further refinement loops are performed</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Number of loops for iterative estimation of </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">P_stable </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>in BAL/STOR (see eq. S9 &amp; explanation below eq. S19). Usually, 2 suffices; use 1 for quicker (but less accurate) simulations.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">This number defines the amount of discrete steps between 0 and </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>max(E_hydro + E_solar + E_wind)</t>
+    </r>
+  </si>
+  <si>
+    <t>[name 1]</t>
+  </si>
+  <si>
+    <t>[name 2]</t>
+  </si>
+  <si>
+    <t>[name 3]</t>
+  </si>
+  <si>
+    <t>set to 1 to plot operational regime statistics, or to 0 to turn off</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">set to 1 to plot regulated reservoir release statistics [see </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_rules_month</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> and </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>plot_rules_hr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> below</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, or to 0 to turn off</t>
     </r>
   </si>
   <si>
@@ -1567,291 +1794,64 @@
         <b/>
         <i/>
         <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[only use if already known from previous run]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> The optimal value in the range of the ELCC for STOR</t>
-    </r>
-  </si>
-  <si>
-    <t>path_inputs</t>
-  </si>
-  <si>
-    <t>path_outputs</t>
-  </si>
-  <si>
-    <t>path to folder with input data sheets</t>
-  </si>
-  <si>
-    <t>path where output will be located</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>parameter</t>
-  </si>
-  <si>
-    <t>explanation</t>
-  </si>
-  <si>
-    <t>value(s)</t>
-  </si>
-  <si>
-    <t>path</t>
-  </si>
-  <si>
-    <t>notes</t>
-  </si>
-  <si>
-    <t>simulation period</t>
-  </si>
-  <si>
-    <t>simulation settings</t>
-  </si>
-  <si>
-    <t>physical constants</t>
-  </si>
-  <si>
-    <t>simulation accuracy</t>
-  </si>
-  <si>
-    <t>years_skip</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">this parameter allows to skip the first </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">year_skip </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>years of the entered data (default: 0)</t>
-    </r>
-  </si>
-  <si>
-    <t>miscellaneous simulation parameters</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">represents number of years of filling as threshold for determining </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>f_reg</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> if left unspecified by user (see sheet "Hydropower plant parameters"). Default/recommended is unity, so</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> f_reg </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>represents the fraction of annual mean inflow that would take exactly one year to fill reservoir.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">When </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>min(Psi)</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> (eq. S21) is lower than this threshold, no further refinement loops are performed</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Number of loops for iterative estimation of </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">P_stable </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>in BAL/STOR (see eq. S9 &amp; explanation below eq. S19). Usually, 2 suffices; use 1 for quicker (but less accurate) simulations.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">This number defines the amount of discrete steps between 0 and </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>max(E_hydro + E_solar + E_wind)</t>
-    </r>
-  </si>
-  <si>
-    <t>[name 1]</t>
-  </si>
-  <si>
-    <t>[name 2]</t>
-  </si>
-  <si>
-    <t>[name 3]</t>
-  </si>
-  <si>
-    <t>set to 1 to plot operational regime statistics, or to 0 to turn off</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">set to 1 to plot regulated reservoir release statistics [see </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>plot_rules_month</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> and </t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>plot_rules_hr</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> below</t>
-    </r>
-    <r>
-      <rPr>
-        <i/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, or to 0 to turn off</t>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[leave empty for zeros]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> name of corresponding worksheet in the "data" Excel sheets (use the "inflow" workbook) from which to pull data on </t>
+    </r>
+    <r>
+      <rPr>
+        <u/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>lateral</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> inflow to a downstream cascade plant (hourly flow in </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>m^3/s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>; hours in rows, years in columns)</t>
     </r>
   </si>
 </sst>
@@ -2478,31 +2478,31 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B1" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>210</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B2" s="18"/>
       <c r="C2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B3" s="18"/>
       <c r="C3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
   </sheetData>
@@ -2534,13 +2534,13 @@
         <v>13</v>
       </c>
       <c r="C2" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D2" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>224</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>225</v>
       </c>
     </row>
     <row r="3" spans="1:5" s="10" customFormat="1" x14ac:dyDescent="0.35">
@@ -2596,12 +2596,12 @@
         <v>176</v>
       </c>
     </row>
-    <row r="10" spans="1:5" s="3" customFormat="1" ht="58" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
       <c r="A10" s="5" t="s">
         <v>108</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>177</v>
+        <v>227</v>
       </c>
     </row>
     <row r="11" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2609,7 +2609,7 @@
         <v>21</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2617,7 +2617,7 @@
         <v>20</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="13" spans="1:5" s="3" customFormat="1" ht="43.5" customHeight="1" x14ac:dyDescent="0.35">
@@ -2625,7 +2625,7 @@
         <v>17</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2633,7 +2633,7 @@
         <v>18</v>
       </c>
       <c r="B14" s="17" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:5" s="3" customFormat="1" ht="43.5" x14ac:dyDescent="0.35">
@@ -2641,7 +2641,7 @@
         <v>19</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:5" s="3" customFormat="1" ht="29" x14ac:dyDescent="0.35">
@@ -2649,7 +2649,7 @@
         <v>22</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="17" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2663,7 +2663,7 @@
         <v>23</v>
       </c>
       <c r="B18" s="17" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="19" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2677,7 +2677,7 @@
         <v>24</v>
       </c>
       <c r="B20" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="21" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2691,7 +2691,7 @@
         <v>29</v>
       </c>
       <c r="B22" s="17" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="23" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2699,7 +2699,7 @@
         <v>27</v>
       </c>
       <c r="B23" s="17" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="24" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2707,7 +2707,7 @@
         <v>26</v>
       </c>
       <c r="B24" s="17" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="25" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2715,7 +2715,7 @@
         <v>25</v>
       </c>
       <c r="B25" s="17" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="26" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2723,7 +2723,7 @@
         <v>30</v>
       </c>
       <c r="B26" s="17" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="27" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2739,7 +2739,7 @@
         <v>33</v>
       </c>
       <c r="B28" s="17" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="29" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2908,10 +2908,10 @@
     </row>
     <row r="50" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A50" s="5" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="51" spans="1:2" s="8" customFormat="1" ht="21" x14ac:dyDescent="0.5">
@@ -2925,7 +2925,7 @@
         <v>59</v>
       </c>
       <c r="B52" s="17" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="53" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2941,7 +2941,7 @@
         <v>61</v>
       </c>
       <c r="B54" s="17" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="55" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -2949,7 +2949,7 @@
         <v>62</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="56" spans="1:2" s="2" customFormat="1" x14ac:dyDescent="0.35">
@@ -3008,10 +3008,10 @@
     </row>
     <row r="63" spans="1:2" s="2" customFormat="1" ht="29" x14ac:dyDescent="0.35">
       <c r="A63" s="5" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -3036,13 +3036,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>207</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -3052,7 +3052,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" s="21" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B3" s="20"/>
       <c r="C3" s="20"/>
@@ -3077,18 +3077,18 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B6" s="22">
         <v>0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A8" s="21" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B8" s="20"/>
       <c r="C8" s="20"/>
@@ -3118,7 +3118,7 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A12" s="21" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B12" s="20"/>
       <c r="C12" s="20"/>
@@ -3147,7 +3147,7 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A16" s="21" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B16" s="20"/>
       <c r="C16" s="20"/>
@@ -3160,7 +3160,7 @@
         <v>1000</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="43.5" x14ac:dyDescent="0.35">
@@ -3171,7 +3171,7 @@
         <v>2</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="19" spans="1:3" ht="29" x14ac:dyDescent="0.35">
@@ -3182,12 +3182,12 @@
         <v>0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A21" s="21" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="20"/>
@@ -3200,7 +3200,7 @@
         <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.35">
@@ -3253,13 +3253,13 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>207</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="C1" s="5" t="s">
-        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -3385,7 +3385,7 @@
       </c>
       <c r="B15" s="23"/>
       <c r="C15" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -3403,16 +3403,16 @@
       </c>
       <c r="B17" s="23"/>
       <c r="C17" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B18" s="23"/>
       <c r="C18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -3460,10 +3460,10 @@
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="2" spans="1:15" x14ac:dyDescent="0.35">
@@ -3637,11 +3637,11 @@
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B30" s="23"/>
       <c r="C30" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
   </sheetData>

</xml_diff>